<commit_message>
Added surrogate Keys to DataMap
</commit_message>
<xml_diff>
--- a/docs/Data Map/Citibike Data Map.xlsx
+++ b/docs/Data Map/Citibike Data Map.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/florentin/Desktop/Entwicklung/Repos/Citibike_Project/docs/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/florentin/Desktop/Entwicklung/Repos/Citibike_Project/docs/Data Map/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A7F73CF8-41C7-EB48-A6F8-0D44980755E8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2A76BF01-14D1-6C4B-8133-2A932BCE378B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="660" windowWidth="30240" windowHeight="17340" xr2:uid="{A950CCA5-45F8-463E-BCD8-1FA9D9B98C57}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="226" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="281" uniqueCount="90">
   <si>
     <t>Target</t>
   </si>
@@ -267,6 +267,45 @@
   </si>
   <si>
     <t>SELECT DISTINCT member_casual AS user_type - Natural Key</t>
+  </si>
+  <si>
+    <t>trip_sk</t>
+  </si>
+  <si>
+    <t>-</t>
+  </si>
+  <si>
+    <t>ROW_NUMBER() OVER (ORDER BY started_at) - Surrogate Key (PK)</t>
+  </si>
+  <si>
+    <t>sation_sk</t>
+  </si>
+  <si>
+    <t>ROW_NUMBER() OVER (ORDER BY station_id) - Surrogate Key (PK)</t>
+  </si>
+  <si>
+    <t>bike_sk</t>
+  </si>
+  <si>
+    <t>date_sk</t>
+  </si>
+  <si>
+    <t>TO_CHAR(date_val, 'YYYYMMDD')::INTEGER - Smart Surrogate Key (PK, z.B. 20240115)</t>
+  </si>
+  <si>
+    <t>ROW_NUMBER() OVER (ORDER BY bike_type) - Surrogate Key (PK)</t>
+  </si>
+  <si>
+    <t>weather_sk</t>
+  </si>
+  <si>
+    <t>ROW_NUMBER() OVER (ORDER BY date_key) - Surrogate Key (PK)</t>
+  </si>
+  <si>
+    <t>user_sk</t>
+  </si>
+  <si>
+    <t>ROW_NUMBER() OVER (ORDER BY user_type) - Surrogate Key (PK)</t>
   </si>
 </sst>
 </file>
@@ -319,7 +358,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="21">
+  <borders count="23">
     <border>
       <left/>
       <right/>
@@ -593,11 +632,35 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="25">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center"/>
@@ -642,6 +705,9 @@
       <alignment horizontal="left" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="19" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="14" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -660,8 +726,11 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="18" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="21" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="22" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -1000,7 +1069,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:J26"/>
+  <dimension ref="A1:J32"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="22.6640625" bestFit="1" customWidth="1"/>
@@ -1015,20 +1084,20 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:10" ht="21" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A1" s="16" t="s">
+      <c r="A1" s="17" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="17"/>
-      <c r="C1" s="17"/>
-      <c r="D1" s="17"/>
-      <c r="E1" s="18"/>
-      <c r="F1" s="19" t="s">
-        <v>1</v>
-      </c>
-      <c r="G1" s="17"/>
-      <c r="H1" s="17"/>
-      <c r="I1" s="18"/>
-      <c r="J1" s="20" t="s">
+      <c r="B1" s="18"/>
+      <c r="C1" s="18"/>
+      <c r="D1" s="18"/>
+      <c r="E1" s="19"/>
+      <c r="F1" s="20" t="s">
+        <v>1</v>
+      </c>
+      <c r="G1" s="18"/>
+      <c r="H1" s="18"/>
+      <c r="I1" s="19"/>
+      <c r="J1" s="21" t="s">
         <v>13</v>
       </c>
     </row>
@@ -1060,17 +1129,17 @@
       <c r="I2" s="6" t="s">
         <v>4</v>
       </c>
-      <c r="J2" s="21"/>
-    </row>
-    <row r="3" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="J2" s="22"/>
+    </row>
+    <row r="3" spans="1:10" ht="16" thickBot="1" x14ac:dyDescent="0.25">
       <c r="A3" s="3" t="s">
         <v>14</v>
       </c>
       <c r="B3" s="2" t="s">
-        <v>15</v>
+        <v>77</v>
       </c>
       <c r="C3" s="2" t="s">
-        <v>16</v>
+        <v>53</v>
       </c>
       <c r="D3" s="2" t="s">
         <v>8</v>
@@ -1085,13 +1154,13 @@
         <v>18</v>
       </c>
       <c r="H3" s="2" t="s">
-        <v>15</v>
+        <v>78</v>
       </c>
       <c r="I3" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="J3" s="12" t="s">
-        <v>19</v>
+        <v>78</v>
+      </c>
+      <c r="J3" s="13" t="s">
+        <v>79</v>
       </c>
     </row>
     <row r="4" spans="1:10" x14ac:dyDescent="0.2">
@@ -1099,10 +1168,10 @@
         <v>14</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="D4" s="2" t="s">
         <v>8</v>
@@ -1117,13 +1186,13 @@
         <v>18</v>
       </c>
       <c r="H4" s="2" t="s">
-        <v>21</v>
+        <v>15</v>
       </c>
       <c r="I4" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="J4" s="13" t="s">
-        <v>22</v>
+        <v>16</v>
+      </c>
+      <c r="J4" s="12" t="s">
+        <v>19</v>
       </c>
     </row>
     <row r="5" spans="1:10" x14ac:dyDescent="0.2">
@@ -1131,10 +1200,10 @@
         <v>14</v>
       </c>
       <c r="B5" s="2" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="C5" s="2" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="D5" s="2" t="s">
         <v>8</v>
@@ -1149,13 +1218,13 @@
         <v>18</v>
       </c>
       <c r="H5" s="2" t="s">
-        <v>23</v>
+        <v>21</v>
       </c>
       <c r="I5" s="1" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="J5" s="13" t="s">
-        <v>24</v>
+        <v>22</v>
       </c>
     </row>
     <row r="6" spans="1:10" x14ac:dyDescent="0.2">
@@ -1163,7 +1232,7 @@
         <v>14</v>
       </c>
       <c r="B6" s="2" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="C6" s="2" t="s">
         <v>16</v>
@@ -1181,7 +1250,7 @@
         <v>18</v>
       </c>
       <c r="H6" s="2" t="s">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="I6" s="1" t="s">
         <v>16</v>
@@ -1195,7 +1264,7 @@
         <v>14</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="C7" s="2" t="s">
         <v>16</v>
@@ -1213,13 +1282,13 @@
         <v>18</v>
       </c>
       <c r="H7" s="2" t="s">
-        <v>27</v>
+        <v>25</v>
       </c>
       <c r="I7" s="1" t="s">
         <v>16</v>
       </c>
       <c r="J7" s="13" t="s">
-        <v>28</v>
+        <v>24</v>
       </c>
     </row>
     <row r="8" spans="1:10" x14ac:dyDescent="0.2">
@@ -1227,7 +1296,7 @@
         <v>14</v>
       </c>
       <c r="B8" s="2" t="s">
-        <v>29</v>
+        <v>26</v>
       </c>
       <c r="C8" s="2" t="s">
         <v>16</v>
@@ -1245,13 +1314,13 @@
         <v>18</v>
       </c>
       <c r="H8" s="2" t="s">
-        <v>30</v>
+        <v>27</v>
       </c>
       <c r="I8" s="1" t="s">
         <v>16</v>
       </c>
       <c r="J8" s="13" t="s">
-        <v>31</v>
+        <v>28</v>
       </c>
     </row>
     <row r="9" spans="1:10" x14ac:dyDescent="0.2">
@@ -1259,10 +1328,10 @@
         <v>14</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>32</v>
+        <v>29</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>33</v>
+        <v>16</v>
       </c>
       <c r="D9" s="2" t="s">
         <v>8</v>
@@ -1277,30 +1346,30 @@
         <v>18</v>
       </c>
       <c r="H9" s="2" t="s">
-        <v>34</v>
+        <v>30</v>
       </c>
       <c r="I9" s="1" t="s">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="J9" s="13" t="s">
-        <v>35</v>
+        <v>31</v>
       </c>
     </row>
     <row r="10" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A10" s="3" t="s">
-        <v>36</v>
+        <v>14</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>37</v>
+        <v>32</v>
       </c>
       <c r="C10" s="2" t="s">
-        <v>16</v>
+        <v>33</v>
       </c>
       <c r="D10" s="2" t="s">
-        <v>12</v>
-      </c>
-      <c r="E10" s="1">
-        <v>1</v>
+        <v>8</v>
+      </c>
+      <c r="E10" s="1" t="s">
+        <v>9</v>
       </c>
       <c r="F10" s="2" t="s">
         <v>17</v>
@@ -1309,24 +1378,24 @@
         <v>18</v>
       </c>
       <c r="H10" s="2" t="s">
-        <v>38</v>
+        <v>34</v>
       </c>
       <c r="I10" s="1" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="J10" s="13" t="s">
-        <v>39</v>
-      </c>
-    </row>
-    <row r="11" spans="1:10" ht="32" x14ac:dyDescent="0.2">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A11" s="3" t="s">
         <v>36</v>
       </c>
       <c r="B11" s="2" t="s">
-        <v>40</v>
+        <v>80</v>
       </c>
       <c r="C11" s="2" t="s">
-        <v>16</v>
+        <v>53</v>
       </c>
       <c r="D11" s="2" t="s">
         <v>12</v>
@@ -1340,14 +1409,14 @@
       <c r="G11" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="H11" s="11" t="s">
-        <v>41</v>
+      <c r="H11" s="2" t="s">
+        <v>78</v>
       </c>
       <c r="I11" s="1" t="s">
-        <v>16</v>
+        <v>78</v>
       </c>
       <c r="J11" s="13" t="s">
-        <v>42</v>
+        <v>81</v>
       </c>
     </row>
     <row r="12" spans="1:10" x14ac:dyDescent="0.2">
@@ -1355,10 +1424,10 @@
         <v>36</v>
       </c>
       <c r="B12" s="2" t="s">
-        <v>43</v>
+        <v>37</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>44</v>
+        <v>16</v>
       </c>
       <c r="D12" s="2" t="s">
         <v>12</v>
@@ -1373,24 +1442,24 @@
         <v>18</v>
       </c>
       <c r="H12" s="2" t="s">
-        <v>45</v>
+        <v>38</v>
       </c>
       <c r="I12" s="1" t="s">
-        <v>44</v>
+        <v>16</v>
       </c>
       <c r="J12" s="13" t="s">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="13" spans="1:10" x14ac:dyDescent="0.2">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="13" spans="1:10" ht="32" x14ac:dyDescent="0.2">
       <c r="A13" s="3" t="s">
         <v>36</v>
       </c>
       <c r="B13" s="2" t="s">
-        <v>47</v>
+        <v>40</v>
       </c>
       <c r="C13" s="2" t="s">
-        <v>44</v>
+        <v>16</v>
       </c>
       <c r="D13" s="2" t="s">
         <v>12</v>
@@ -1404,25 +1473,25 @@
       <c r="G13" s="2" t="s">
         <v>18</v>
       </c>
-      <c r="H13" s="2" t="s">
-        <v>48</v>
+      <c r="H13" s="11" t="s">
+        <v>41</v>
       </c>
       <c r="I13" s="1" t="s">
-        <v>44</v>
+        <v>16</v>
       </c>
       <c r="J13" s="13" t="s">
-        <v>49</v>
+        <v>42</v>
       </c>
     </row>
     <row r="14" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A14" s="3" t="s">
-        <v>50</v>
+        <v>36</v>
       </c>
       <c r="B14" s="2" t="s">
-        <v>20</v>
+        <v>43</v>
       </c>
       <c r="C14" s="2" t="s">
-        <v>11</v>
+        <v>44</v>
       </c>
       <c r="D14" s="2" t="s">
         <v>12</v>
@@ -1437,24 +1506,24 @@
         <v>18</v>
       </c>
       <c r="H14" s="2" t="s">
-        <v>34</v>
+        <v>45</v>
       </c>
       <c r="I14" s="1" t="s">
-        <v>10</v>
+        <v>44</v>
       </c>
       <c r="J14" s="13" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
     </row>
     <row r="15" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A15" s="3" t="s">
-        <v>50</v>
+        <v>36</v>
       </c>
       <c r="B15" s="2" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>53</v>
+        <v>44</v>
       </c>
       <c r="D15" s="2" t="s">
         <v>12</v>
@@ -1469,13 +1538,13 @@
         <v>18</v>
       </c>
       <c r="H15" s="2" t="s">
-        <v>34</v>
+        <v>48</v>
       </c>
       <c r="I15" s="1" t="s">
-        <v>10</v>
+        <v>44</v>
       </c>
       <c r="J15" s="13" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
     </row>
     <row r="16" spans="1:10" x14ac:dyDescent="0.2">
@@ -1483,7 +1552,7 @@
         <v>50</v>
       </c>
       <c r="B16" s="2" t="s">
-        <v>55</v>
+        <v>83</v>
       </c>
       <c r="C16" s="2" t="s">
         <v>53</v>
@@ -1507,7 +1576,7 @@
         <v>10</v>
       </c>
       <c r="J16" s="13" t="s">
-        <v>56</v>
+        <v>84</v>
       </c>
     </row>
     <row r="17" spans="1:10" x14ac:dyDescent="0.2">
@@ -1515,10 +1584,10 @@
         <v>50</v>
       </c>
       <c r="B17" s="2" t="s">
-        <v>57</v>
+        <v>20</v>
       </c>
       <c r="C17" s="2" t="s">
-        <v>53</v>
+        <v>11</v>
       </c>
       <c r="D17" s="2" t="s">
         <v>12</v>
@@ -1539,7 +1608,7 @@
         <v>10</v>
       </c>
       <c r="J17" s="13" t="s">
-        <v>58</v>
+        <v>51</v>
       </c>
     </row>
     <row r="18" spans="1:10" x14ac:dyDescent="0.2">
@@ -1547,10 +1616,10 @@
         <v>50</v>
       </c>
       <c r="B18" s="2" t="s">
-        <v>59</v>
+        <v>52</v>
       </c>
       <c r="C18" s="2" t="s">
-        <v>16</v>
+        <v>53</v>
       </c>
       <c r="D18" s="2" t="s">
         <v>12</v>
@@ -1571,18 +1640,18 @@
         <v>10</v>
       </c>
       <c r="J18" s="13" t="s">
-        <v>60</v>
+        <v>54</v>
       </c>
     </row>
     <row r="19" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A19" s="3" t="s">
-        <v>61</v>
+        <v>50</v>
       </c>
       <c r="B19" s="2" t="s">
-        <v>26</v>
+        <v>55</v>
       </c>
       <c r="C19" s="2" t="s">
-        <v>16</v>
+        <v>53</v>
       </c>
       <c r="D19" s="2" t="s">
         <v>12</v>
@@ -1597,24 +1666,24 @@
         <v>18</v>
       </c>
       <c r="H19" s="2" t="s">
-        <v>27</v>
+        <v>34</v>
       </c>
       <c r="I19" s="1" t="s">
-        <v>16</v>
+        <v>10</v>
       </c>
       <c r="J19" s="13" t="s">
-        <v>62</v>
+        <v>56</v>
       </c>
     </row>
     <row r="20" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A20" s="3" t="s">
-        <v>63</v>
+        <v>50</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>20</v>
+        <v>57</v>
       </c>
       <c r="C20" s="2" t="s">
-        <v>11</v>
+        <v>53</v>
       </c>
       <c r="D20" s="2" t="s">
         <v>12</v>
@@ -1626,27 +1695,27 @@
         <v>17</v>
       </c>
       <c r="G20" s="2" t="s">
-        <v>64</v>
+        <v>18</v>
       </c>
       <c r="H20" s="2" t="s">
-        <v>20</v>
+        <v>34</v>
       </c>
       <c r="I20" s="1" t="s">
-        <v>65</v>
+        <v>10</v>
       </c>
       <c r="J20" s="13" t="s">
-        <v>66</v>
+        <v>58</v>
       </c>
     </row>
     <row r="21" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A21" s="3" t="s">
-        <v>63</v>
+        <v>50</v>
       </c>
       <c r="B21" s="2" t="s">
-        <v>67</v>
+        <v>59</v>
       </c>
       <c r="C21" s="2" t="s">
-        <v>44</v>
+        <v>16</v>
       </c>
       <c r="D21" s="2" t="s">
         <v>12</v>
@@ -1658,27 +1727,27 @@
         <v>17</v>
       </c>
       <c r="G21" s="2" t="s">
-        <v>64</v>
+        <v>18</v>
       </c>
       <c r="H21" s="2" t="s">
-        <v>67</v>
+        <v>34</v>
       </c>
       <c r="I21" s="1" t="s">
-        <v>44</v>
+        <v>10</v>
       </c>
       <c r="J21" s="13" t="s">
-        <v>68</v>
+        <v>60</v>
       </c>
     </row>
     <row r="22" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A22" s="3" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B22" s="2" t="s">
-        <v>69</v>
+        <v>82</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>44</v>
+        <v>53</v>
       </c>
       <c r="D22" s="2" t="s">
         <v>12</v>
@@ -1690,27 +1759,27 @@
         <v>17</v>
       </c>
       <c r="G22" s="2" t="s">
-        <v>64</v>
+        <v>18</v>
       </c>
       <c r="H22" s="2" t="s">
-        <v>69</v>
+        <v>78</v>
       </c>
       <c r="I22" s="1" t="s">
-        <v>44</v>
+        <v>78</v>
       </c>
       <c r="J22" s="13" t="s">
-        <v>70</v>
+        <v>85</v>
       </c>
     </row>
     <row r="23" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A23" s="3" t="s">
-        <v>63</v>
+        <v>61</v>
       </c>
       <c r="B23" s="2" t="s">
-        <v>71</v>
+        <v>26</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>44</v>
+        <v>16</v>
       </c>
       <c r="D23" s="2" t="s">
         <v>12</v>
@@ -1722,32 +1791,32 @@
         <v>17</v>
       </c>
       <c r="G23" s="2" t="s">
-        <v>64</v>
+        <v>18</v>
       </c>
       <c r="H23" s="2" t="s">
-        <v>71</v>
+        <v>27</v>
       </c>
       <c r="I23" s="1" t="s">
-        <v>44</v>
+        <v>16</v>
       </c>
       <c r="J23" s="13" t="s">
-        <v>72</v>
-      </c>
-    </row>
-    <row r="24" spans="1:10" ht="48" x14ac:dyDescent="0.2">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="24" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A24" s="3" t="s">
         <v>63</v>
       </c>
       <c r="B24" s="2" t="s">
-        <v>73</v>
+        <v>86</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>16</v>
+        <v>53</v>
       </c>
       <c r="D24" s="2" t="s">
         <v>12</v>
       </c>
-      <c r="E24" s="14">
+      <c r="E24" s="1">
         <v>1</v>
       </c>
       <c r="F24" s="2" t="s">
@@ -1757,50 +1826,242 @@
         <v>64</v>
       </c>
       <c r="H24" s="2" t="s">
+        <v>78</v>
+      </c>
+      <c r="I24" s="1" t="s">
+        <v>78</v>
+      </c>
+      <c r="J24" s="13" t="s">
+        <v>87</v>
+      </c>
+    </row>
+    <row r="25" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A25" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="C25" s="2" t="s">
+        <v>11</v>
+      </c>
+      <c r="D25" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E25" s="1">
+        <v>1</v>
+      </c>
+      <c r="F25" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G25" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="H25" s="2" t="s">
+        <v>20</v>
+      </c>
+      <c r="I25" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="J25" s="13" t="s">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A26" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="C26" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="D26" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E26" s="1">
+        <v>1</v>
+      </c>
+      <c r="F26" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G26" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="H26" s="2" t="s">
+        <v>67</v>
+      </c>
+      <c r="I26" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="J26" s="13" t="s">
+        <v>68</v>
+      </c>
+    </row>
+    <row r="27" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A27" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="C27" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="D27" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E27" s="1">
+        <v>1</v>
+      </c>
+      <c r="F27" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G27" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="H27" s="2" t="s">
+        <v>69</v>
+      </c>
+      <c r="I27" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="J27" s="13" t="s">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="28" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="A28" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="B28" s="2" t="s">
         <v>71</v>
       </c>
-      <c r="I24" s="1" t="s">
+      <c r="C28" s="2" t="s">
         <v>44</v>
       </c>
-      <c r="J24" s="22" t="s">
+      <c r="D28" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E28" s="1">
+        <v>1</v>
+      </c>
+      <c r="F28" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G28" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="H28" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="I28" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="J28" s="13" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="29" spans="1:10" ht="48" x14ac:dyDescent="0.2">
+      <c r="A29" s="3" t="s">
+        <v>63</v>
+      </c>
+      <c r="B29" s="2" t="s">
+        <v>73</v>
+      </c>
+      <c r="C29" s="2" t="s">
+        <v>16</v>
+      </c>
+      <c r="D29" s="2" t="s">
+        <v>12</v>
+      </c>
+      <c r="E29" s="14">
+        <v>1</v>
+      </c>
+      <c r="F29" s="2" t="s">
+        <v>17</v>
+      </c>
+      <c r="G29" s="2" t="s">
+        <v>64</v>
+      </c>
+      <c r="H29" s="2" t="s">
+        <v>71</v>
+      </c>
+      <c r="I29" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="J29" s="16" t="s">
         <v>74</v>
       </c>
     </row>
-    <row r="25" spans="1:10" ht="16" thickBot="1" x14ac:dyDescent="0.25">
-      <c r="A25" s="9" t="s">
+    <row r="30" spans="1:10" ht="16" x14ac:dyDescent="0.2">
+      <c r="A30" s="23" t="s">
         <v>75</v>
       </c>
-      <c r="B25" s="10" t="s">
+      <c r="B30" s="24" t="s">
+        <v>88</v>
+      </c>
+      <c r="C30" s="24" t="s">
+        <v>53</v>
+      </c>
+      <c r="D30" s="24" t="s">
+        <v>12</v>
+      </c>
+      <c r="E30" s="14">
+        <v>1</v>
+      </c>
+      <c r="F30" s="24" t="s">
+        <v>17</v>
+      </c>
+      <c r="G30" s="24" t="s">
+        <v>18</v>
+      </c>
+      <c r="H30" s="24" t="s">
+        <v>78</v>
+      </c>
+      <c r="I30" s="14" t="s">
+        <v>78</v>
+      </c>
+      <c r="J30" s="16" t="s">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="31" spans="1:10" ht="16" thickBot="1" x14ac:dyDescent="0.25">
+      <c r="A31" s="9" t="s">
+        <v>75</v>
+      </c>
+      <c r="B31" s="10" t="s">
         <v>29</v>
       </c>
-      <c r="C25" s="10" t="s">
+      <c r="C31" s="10" t="s">
         <v>16</v>
       </c>
-      <c r="D25" s="10" t="s">
+      <c r="D31" s="10" t="s">
         <v>12</v>
       </c>
-      <c r="E25" s="14">
-        <v>1</v>
-      </c>
-      <c r="F25" s="10" t="s">
-        <v>17</v>
-      </c>
-      <c r="G25" s="10" t="s">
-        <v>18</v>
-      </c>
-      <c r="H25" s="10" t="s">
+      <c r="E31" s="14">
+        <v>1</v>
+      </c>
+      <c r="F31" s="10" t="s">
+        <v>17</v>
+      </c>
+      <c r="G31" s="10" t="s">
+        <v>18</v>
+      </c>
+      <c r="H31" s="10" t="s">
         <v>30</v>
       </c>
-      <c r="I25" s="14" t="s">
+      <c r="I31" s="14" t="s">
         <v>16</v>
       </c>
-      <c r="J25" s="10" t="s">
+      <c r="J31" s="10" t="s">
         <v>76</v>
       </c>
     </row>
-    <row r="26" spans="1:10" x14ac:dyDescent="0.2">
-      <c r="E26" s="15"/>
-      <c r="I26" s="15"/>
+    <row r="32" spans="1:10" x14ac:dyDescent="0.2">
+      <c r="E32" s="15"/>
+      <c r="I32" s="15"/>
     </row>
   </sheetData>
   <mergeCells count="3">

</xml_diff>